<commit_message>
organização direção e estatutos em modelo novo
</commit_message>
<xml_diff>
--- a/DRIVE/1. Direção/2. Financeiro/2.2 Contabilidade/Compras propostas/Proposta SoftRoutine - PA JBL/Divisão de compra.xlsx
+++ b/DRIVE/1. Direção/2. Financeiro/2.2 Contabilidade/Compras propostas/Proposta SoftRoutine - PA JBL/Divisão de compra.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruisa\mind7\MINDSET\DRIVE\1. Direção\2. Financeiro\2.2 Contabilidade\Compras\Proposta SR - PA JBL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ruisa\mind7\MINDSET\DRIVE\1. Direção\2. Financeiro\2.2 Contabilidade\Compras propostas\Proposta SoftRoutine - PA JBL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35573709-BBBD-4F53-8ECA-37117A9DF79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C532E8-E2C3-4A56-8758-87F5725331FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9FEF305E-DE7E-4357-B4A2-9AE6791F5EA4}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11424" windowHeight="13776" xr2:uid="{9FEF305E-DE7E-4357-B4A2-9AE6791F5EA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
   <si>
     <t>Rui Alves</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>valor a pagar aos investidores</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Inês César</t>
   </si>
 </sst>
 </file>
@@ -450,11 +456,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{039C83DE-24BC-430E-B8A4-170A66031777}">
-  <dimension ref="G7:L14"/>
+  <dimension ref="G7:L15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
@@ -489,7 +496,7 @@
       </c>
       <c r="L8">
         <f>SUM(H8:H16)</f>
-        <v>1585</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="9" spans="7:12" x14ac:dyDescent="0.3">
@@ -500,7 +507,7 @@
         <v>200</v>
       </c>
       <c r="I9">
-        <f t="shared" ref="I9:I14" si="0">H9*1.5</f>
+        <f t="shared" ref="I9:I15" si="0">H9*1.5</f>
         <v>300</v>
       </c>
       <c r="K9" t="s">
@@ -508,7 +515,7 @@
       </c>
       <c r="L9">
         <f>SUM(I8:I14)</f>
-        <v>2377.5</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="10" spans="7:12" x14ac:dyDescent="0.3">
@@ -522,6 +529,9 @@
         <f t="shared" si="0"/>
         <v>225</v>
       </c>
+      <c r="J10" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="11" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G11" t="s">
@@ -540,15 +550,18 @@
         <v>4</v>
       </c>
       <c r="H12">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="I12">
         <f t="shared" si="0"/>
-        <v>577.5</v>
+        <v>600</v>
+      </c>
+      <c r="J12" t="s">
+        <v>12</v>
       </c>
       <c r="L12">
         <f>L9/6</f>
-        <v>396.25</v>
+        <v>375</v>
       </c>
     </row>
     <row r="13" spans="7:12" x14ac:dyDescent="0.3">
@@ -562,17 +575,38 @@
         <f t="shared" si="0"/>
         <v>525</v>
       </c>
+      <c r="J13" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G14" t="s">
         <v>8</v>
       </c>
       <c r="H14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I14">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>150</v>
+      </c>
+      <c r="J14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" x14ac:dyDescent="0.3">
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15">
+        <v>100</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="J15" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>